<commit_message>
Added Kira's feedback for HA Pairs
</commit_message>
<xml_diff>
--- a/data/PROTECT_Hazard_Asset_Pairs_KR.xlsx
+++ b/data/PROTECT_Hazard_Asset_Pairs_KR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amcclary\Documents\GitHub\PROTECT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E80D1B6D-C9C1-4C57-8EA7-4B077AB04436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C395D10-03DD-4410-B512-01E83B3E6041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{84747710-1B95-4224-8C27-75ECDD8FBEBA}"/>
   </bookViews>
@@ -39,12 +39,12 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={1058747B-8F6C-46D6-AD19-E5B4A738E505}</author>
+    <author>tc={F696103D-7C9F-4441-A1F7-95B1F8A69670}</author>
+    <author>tc={A0230801-4CCA-4581-8FB5-13FF5D469B46}</author>
     <author>tc={C47A4326-D46A-463A-A8F0-5D5A2D06D446}</author>
-    <author>tc={A0230801-4CCA-4581-8FB5-13FF5D469B46}</author>
-    <author>tc={F696103D-7C9F-4441-A1F7-95B1F8A69670}</author>
   </authors>
   <commentList>
-    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{1058747B-8F6C-46D6-AD19-E5B4A738E505}">
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{1058747B-8F6C-46D6-AD19-E5B4A738E505}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -52,15 +52,15 @@
     I’m not sure how much an avalanche would physically damage a roadway, unless concrete slopes, etc. are considered as part of the roadway infrastructure, in which case ignore this comment. </t>
       </text>
     </comment>
-    <comment ref="C13" authorId="1" shapeId="0" xr:uid="{C47A4326-D46A-463A-A8F0-5D5A2D06D446}">
+    <comment ref="B11" authorId="1" shapeId="0" xr:uid="{F696103D-7C9F-4441-A1F7-95B1F8A69670}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    I don’t think bus stops are worth analyzing, but transit centers should be. And maybe we also include the bus maintenance facilities here since all of the bus assets would be stored here. This could include school district bus yards too or any other fleet yard</t>
+    I don’t think I understand what a debris flow is. How is this different from a landslide?</t>
       </text>
     </comment>
-    <comment ref="C14" authorId="2" shapeId="0" xr:uid="{A0230801-4CCA-4581-8FB5-13FF5D469B46}">
+    <comment ref="C15" authorId="2" shapeId="0" xr:uid="{A0230801-4CCA-4581-8FB5-13FF5D469B46}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -68,12 +68,12 @@
     I would think this might be the only time we’d rely on marinas for transportation during an emergency, so this might be the only important hazard to assess for marinas</t>
       </text>
     </comment>
-    <comment ref="B15" authorId="3" shapeId="0" xr:uid="{F696103D-7C9F-4441-A1F7-95B1F8A69670}">
+    <comment ref="C18" authorId="3" shapeId="0" xr:uid="{C47A4326-D46A-463A-A8F0-5D5A2D06D446}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    I don’t think I understand what a debris flow is. How is this different from a landslide?</t>
+    I don’t think bus stops are worth analyzing, but transit centers should be. And maybe we also include the bus maintenance facilities here since all of the bus assets would be stored here. This could include school district bus yards too or any other fleet yard</t>
       </text>
     </comment>
   </commentList>
@@ -1245,23 +1245,24 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="D6" dT="2026-05-28T16:36:33.92" personId="{35A4CF63-5D44-4AFA-9A4F-3509E27DC5C9}" id="{1058747B-8F6C-46D6-AD19-E5B4A738E505}">
+  <threadedComment ref="D3" dT="2026-05-28T16:36:33.92" personId="{35A4CF63-5D44-4AFA-9A4F-3509E27DC5C9}" id="{1058747B-8F6C-46D6-AD19-E5B4A738E505}">
     <text xml:space="preserve">I’m not sure how much an avalanche would physically damage a roadway, unless concrete slopes, etc. are considered as part of the roadway infrastructure, in which case ignore this comment. </text>
   </threadedComment>
-  <threadedComment ref="C13" dT="2026-05-28T16:49:11.80" personId="{35A4CF63-5D44-4AFA-9A4F-3509E27DC5C9}" id="{C47A4326-D46A-463A-A8F0-5D5A2D06D446}">
-    <text>I don’t think bus stops are worth analyzing, but transit centers should be. And maybe we also include the bus maintenance facilities here since all of the bus assets would be stored here. This could include school district bus yards too or any other fleet yard</text>
+  <threadedComment ref="B11" dT="2026-05-28T17:40:12.13" personId="{35A4CF63-5D44-4AFA-9A4F-3509E27DC5C9}" id="{F696103D-7C9F-4441-A1F7-95B1F8A69670}">
+    <text>I don’t think I understand what a debris flow is. How is this different from a landslide?</text>
   </threadedComment>
-  <threadedComment ref="C14" dT="2026-05-28T16:51:56.34" personId="{35A4CF63-5D44-4AFA-9A4F-3509E27DC5C9}" id="{A0230801-4CCA-4581-8FB5-13FF5D469B46}">
+  <threadedComment ref="C15" dT="2026-05-28T16:51:56.34" personId="{35A4CF63-5D44-4AFA-9A4F-3509E27DC5C9}" id="{A0230801-4CCA-4581-8FB5-13FF5D469B46}">
     <text>I would think this might be the only time we’d rely on marinas for transportation during an emergency, so this might be the only important hazard to assess for marinas</text>
   </threadedComment>
-  <threadedComment ref="B15" dT="2026-05-28T17:40:12.13" personId="{35A4CF63-5D44-4AFA-9A4F-3509E27DC5C9}" id="{F696103D-7C9F-4441-A1F7-95B1F8A69670}">
-    <text>I don’t think I understand what a debris flow is. How is this different from a landslide?</text>
+  <threadedComment ref="C18" dT="2026-05-28T16:49:11.80" personId="{35A4CF63-5D44-4AFA-9A4F-3509E27DC5C9}" id="{C47A4326-D46A-463A-A8F0-5D5A2D06D446}">
+    <text>I don’t think bus stops are worth analyzing, but transit centers should be. And maybe we also include the bus maintenance facilities here since all of the bus assets would be stored here. This could include school district bus yards too or any other fleet yard</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FAB3A0C-EDE5-4340-ADAC-A1D07AFB6CC5}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1303,56 +1304,52 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="A2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="10"/>
+      <c r="E2" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="10" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>11</v>
+      <c r="D3" s="6" t="s">
+        <v>28</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="I3" s="10" t="s">
         <v>84</v>
@@ -1360,10 +1357,10 @@
     </row>
     <row r="4" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>22</v>
@@ -1372,30 +1369,30 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>23</v>
+        <v>58</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>11</v>
@@ -1411,66 +1408,66 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="2" t="s">
+      <c r="A6" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
+      <c r="F7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="I7" s="10" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>11</v>
@@ -1479,27 +1476,27 @@
         <v>12</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="38.25" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>11</v>
@@ -1508,17 +1505,15 @@
         <v>12</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>84</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="I9" s="10"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
@@ -1543,90 +1538,100 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" ht="38.25" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="I11" s="10"/>
+    </row>
+    <row r="12" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="I11" s="10" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="F12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="10" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
+      <c r="E13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>42</v>
+      </c>
       <c r="I13" s="10" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>45</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>11</v>
@@ -1638,42 +1643,38 @@
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
       <c r="I14" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="10" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="I15" s="10"/>
     </row>
     <row r="16" spans="1:9" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>17</v>
@@ -1682,28 +1683,30 @@
         <v>11</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="I16" s="10"/>
-    </row>
-    <row r="17" spans="1:9" ht="25.5" x14ac:dyDescent="0.2">
+        <v>48</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="25.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>11</v>
@@ -1712,27 +1715,25 @@
         <v>33</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I17" s="10" t="s">
-        <v>85</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="I17" s="10"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>17</v>
+        <v>76</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>11</v>
@@ -1744,7 +1745,7 @@
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
       <c r="I18" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
@@ -1777,55 +1778,55 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F21" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G21" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="H21" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="I20" s="10" t="s">
+      <c r="I21" s="10" t="s">
         <v>84</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A21" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="10" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
@@ -1852,7 +1853,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I22" xr:uid="{3FAB3A0C-EDE5-4340-ADAC-A1D07AFB6CC5}"/>
+  <autoFilter ref="A1:I22" xr:uid="{3FAB3A0C-EDE5-4340-ADAC-A1D07AFB6CC5}">
+    <filterColumn colId="8">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I22">
+      <sortCondition ref="B1:B22"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Simplified Hazard Asset Pairs and dataset list in index.html
</commit_message>
<xml_diff>
--- a/data/PROTECT_Hazard_Asset_Pairs_KR.xlsx
+++ b/data/PROTECT_Hazard_Asset_Pairs_KR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amcclary\Documents\GitHub\PROTECT\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C395D10-03DD-4410-B512-01E83B3E6041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD9CC92A-3B24-49BF-8258-6504498E6431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{84747710-1B95-4224-8C27-75ECDD8FBEBA}"/>
   </bookViews>
@@ -1303,7 +1303,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="38.25" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>32</v>
       </c>
@@ -1326,7 +1326,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="38.25" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>26</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -1459,7 +1459,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" ht="38.25" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>16</v>
       </c>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>43</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>39</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>79</v>
       </c>
@@ -1669,7 +1669,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="25.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>44</v>
       </c>
@@ -1725,7 +1725,7 @@
       </c>
       <c r="I17" s="10"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>80</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="38.25" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>62</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="38.25" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>77</v>
       </c>
@@ -1855,9 +1855,9 @@
   </sheetData>
   <autoFilter ref="A1:I22" xr:uid="{3FAB3A0C-EDE5-4340-ADAC-A1D07AFB6CC5}">
     <filterColumn colId="8">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
+      <filters>
+        <filter val="Maybe"/>
+      </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I22">
       <sortCondition ref="B1:B22"/>

</xml_diff>